<commit_message>
Otomatik Veri Güncellemesi: Excel ve Yönetici Paneli Logları [Nispi Veri]
</commit_message>
<xml_diff>
--- a/Gorev-Listesi.xlsx
+++ b/Gorev-Listesi.xlsx
@@ -20,11 +20,12 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <webPublishing css="0" allowPng="1" codePage="1252"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="109">
   <si>
     <t>CUMA</t>
   </si>
@@ -341,10 +342,16 @@
     <t>???</t>
   </si>
   <si>
-    <t>S.CÜREBAL.</t>
-  </si>
-  <si>
     <t>F.BOZKURT.</t>
+  </si>
+  <si>
+    <t>E.KOL.</t>
+  </si>
+  <si>
+    <t>S.ARAS.</t>
+  </si>
+  <si>
+    <t>A.C.PEHLİVAN.</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1393,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1644,6 +1651,15 @@
     <xf numFmtId="49" fontId="11" fillId="7" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="39" fillId="9" borderId="11" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="9" borderId="12" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="9" borderId="13" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1665,25 +1681,67 @@
     <xf numFmtId="49" fontId="40" fillId="7" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="11" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="12" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="14" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="15" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="16" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="8" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="6" borderId="8" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="6" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="11" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="12" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="13" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="11" xfId="57" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="12" xfId="57" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="13" xfId="57" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="40" fillId="7" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="40" fillId="7" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="11" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="17" xfId="57" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="12" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="18" xfId="57" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="13" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="9" borderId="19" xfId="57" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1752,12 +1810,6 @@
     <xf numFmtId="49" fontId="7" fillId="9" borderId="19" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="14" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="15" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="39" fillId="9" borderId="17" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1767,12 +1819,6 @@
     <xf numFmtId="49" fontId="39" fillId="9" borderId="19" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="8" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="9" borderId="14" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1807,15 +1853,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="9" borderId="19" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="9" borderId="11" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="9" borderId="12" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="9" borderId="13" xfId="57" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2267,65 +2304,65 @@
   <sheetData>
     <row r="1" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="12"/>
-      <c r="B1" s="111" t="s">
+      <c r="B1" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
+      <c r="C1" s="129"/>
+      <c r="D1" s="129"/>
       <c r="E1" s="10"/>
-      <c r="F1" s="112" t="s">
+      <c r="F1" s="129" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
+      <c r="G1" s="129"/>
+      <c r="H1" s="129"/>
       <c r="I1" s="10"/>
-      <c r="J1" s="112" t="s">
+      <c r="J1" s="129" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="112"/>
-      <c r="L1" s="113"/>
+      <c r="K1" s="129"/>
+      <c r="L1" s="130"/>
       <c r="M1" s="12"/>
-      <c r="N1" s="116" t="s">
+      <c r="N1" s="133" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
+      <c r="O1" s="127"/>
+      <c r="P1" s="127"/>
       <c r="Q1" s="1"/>
-      <c r="R1" s="110" t="s">
+      <c r="R1" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="110"/>
-      <c r="T1" s="110"/>
+      <c r="S1" s="127"/>
+      <c r="T1" s="127"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="110" t="s">
+      <c r="V1" s="127" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="110"/>
-      <c r="X1" s="110"/>
+      <c r="W1" s="127"/>
+      <c r="X1" s="127"/>
       <c r="Y1" s="1"/>
-      <c r="Z1" s="110" t="s">
+      <c r="Z1" s="127" t="s">
         <v>6</v>
       </c>
-      <c r="AA1" s="110"/>
-      <c r="AB1" s="110"/>
+      <c r="AA1" s="127"/>
+      <c r="AB1" s="127"/>
       <c r="AC1" s="1"/>
-      <c r="AD1" s="110" t="s">
+      <c r="AD1" s="127" t="s">
         <v>0</v>
       </c>
-      <c r="AE1" s="110"/>
-      <c r="AF1" s="110"/>
+      <c r="AE1" s="127"/>
+      <c r="AF1" s="127"/>
       <c r="AG1" s="1"/>
-      <c r="AH1" s="110" t="s">
+      <c r="AH1" s="127" t="s">
         <v>1</v>
       </c>
-      <c r="AI1" s="110"/>
-      <c r="AJ1" s="110"/>
+      <c r="AI1" s="127"/>
+      <c r="AJ1" s="127"/>
       <c r="AK1" s="1"/>
-      <c r="AL1" s="110" t="s">
+      <c r="AL1" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="AM1" s="110"/>
-      <c r="AN1" s="120"/>
+      <c r="AM1" s="127"/>
+      <c r="AN1" s="137"/>
       <c r="AO1" s="12"/>
       <c r="AP1" s="12"/>
       <c r="AQ1" s="12"/>
@@ -2333,74 +2370,74 @@
     </row>
     <row r="2" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
-      <c r="B2" s="114">
+      <c r="B2" s="131">
         <f>N2-3</f>
         <v>46276</v>
       </c>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
+      <c r="C2" s="132"/>
+      <c r="D2" s="132"/>
       <c r="E2" s="11"/>
-      <c r="F2" s="115">
+      <c r="F2" s="132">
         <f>N2-2</f>
         <v>46277</v>
       </c>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
+      <c r="G2" s="132"/>
+      <c r="H2" s="132"/>
       <c r="I2" s="11"/>
-      <c r="J2" s="115">
+      <c r="J2" s="132">
         <f>N2-1</f>
         <v>46278</v>
       </c>
-      <c r="K2" s="115"/>
-      <c r="L2" s="118"/>
+      <c r="K2" s="132"/>
+      <c r="L2" s="135"/>
       <c r="M2" s="12"/>
-      <c r="N2" s="117">
+      <c r="N2" s="134">
         <v>46279</v>
       </c>
-      <c r="O2" s="109"/>
-      <c r="P2" s="109"/>
+      <c r="O2" s="126"/>
+      <c r="P2" s="126"/>
       <c r="Q2" s="53"/>
-      <c r="R2" s="109">
+      <c r="R2" s="126">
         <f>N2+1</f>
         <v>46280</v>
       </c>
-      <c r="S2" s="109"/>
-      <c r="T2" s="109"/>
+      <c r="S2" s="126"/>
+      <c r="T2" s="126"/>
       <c r="U2" s="53"/>
-      <c r="V2" s="109">
+      <c r="V2" s="126">
         <f>N2+2</f>
         <v>46281</v>
       </c>
-      <c r="W2" s="109"/>
-      <c r="X2" s="109"/>
+      <c r="W2" s="126"/>
+      <c r="X2" s="126"/>
       <c r="Y2" s="53"/>
-      <c r="Z2" s="109">
+      <c r="Z2" s="126">
         <f>N2+3</f>
         <v>46282</v>
       </c>
-      <c r="AA2" s="109"/>
-      <c r="AB2" s="109"/>
+      <c r="AA2" s="126"/>
+      <c r="AB2" s="126"/>
       <c r="AC2" s="53"/>
-      <c r="AD2" s="109">
+      <c r="AD2" s="126">
         <f>N2+4</f>
         <v>46283</v>
       </c>
-      <c r="AE2" s="109"/>
-      <c r="AF2" s="109"/>
+      <c r="AE2" s="126"/>
+      <c r="AF2" s="126"/>
       <c r="AG2" s="53"/>
-      <c r="AH2" s="109">
+      <c r="AH2" s="126">
         <f>N2+5</f>
         <v>46284</v>
       </c>
-      <c r="AI2" s="109"/>
-      <c r="AJ2" s="109"/>
+      <c r="AI2" s="126"/>
+      <c r="AJ2" s="126"/>
       <c r="AK2" s="53"/>
-      <c r="AL2" s="109">
+      <c r="AL2" s="126">
         <f>N2+6</f>
         <v>46285</v>
       </c>
-      <c r="AM2" s="109"/>
-      <c r="AN2" s="121"/>
+      <c r="AM2" s="126"/>
+      <c r="AN2" s="138"/>
       <c r="AO2" s="12"/>
       <c r="AP2" s="12"/>
       <c r="AQ2" s="12"/>
@@ -2454,47 +2491,47 @@
     </row>
     <row r="4" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="12"/>
-      <c r="B4" s="119"/>
-      <c r="C4" s="119"/>
-      <c r="D4" s="119"/>
-      <c r="E4" s="119"/>
-      <c r="F4" s="119"/>
-      <c r="G4" s="119"/>
-      <c r="H4" s="119"/>
-      <c r="I4" s="119"/>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="119"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
+      <c r="K4" s="136"/>
+      <c r="L4" s="136"/>
       <c r="M4" s="14"/>
-      <c r="N4" s="99" t="s">
+      <c r="N4" s="102" t="s">
         <v>38</v>
       </c>
-      <c r="O4" s="99"/>
-      <c r="P4" s="99"/>
-      <c r="Q4" s="99"/>
-      <c r="R4" s="99"/>
-      <c r="S4" s="99"/>
-      <c r="T4" s="99"/>
-      <c r="U4" s="99"/>
-      <c r="V4" s="99"/>
-      <c r="W4" s="99"/>
-      <c r="X4" s="99"/>
-      <c r="Y4" s="99"/>
-      <c r="Z4" s="99"/>
-      <c r="AA4" s="99"/>
-      <c r="AB4" s="99"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
+      <c r="T4" s="102"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="102"/>
+      <c r="X4" s="102"/>
+      <c r="Y4" s="102"/>
+      <c r="Z4" s="102"/>
+      <c r="AA4" s="102"/>
+      <c r="AB4" s="102"/>
       <c r="AC4" s="33"/>
-      <c r="AD4" s="119"/>
-      <c r="AE4" s="119"/>
-      <c r="AF4" s="119"/>
-      <c r="AG4" s="119"/>
-      <c r="AH4" s="119"/>
-      <c r="AI4" s="119"/>
-      <c r="AJ4" s="119"/>
-      <c r="AK4" s="119"/>
-      <c r="AL4" s="119"/>
-      <c r="AM4" s="119"/>
-      <c r="AN4" s="119"/>
+      <c r="AD4" s="136"/>
+      <c r="AE4" s="136"/>
+      <c r="AF4" s="136"/>
+      <c r="AG4" s="136"/>
+      <c r="AH4" s="136"/>
+      <c r="AI4" s="136"/>
+      <c r="AJ4" s="136"/>
+      <c r="AK4" s="136"/>
+      <c r="AL4" s="136"/>
+      <c r="AM4" s="136"/>
+      <c r="AN4" s="136"/>
       <c r="AO4" s="12"/>
       <c r="AP4" s="12"/>
       <c r="AQ4" s="12"/>
@@ -2502,45 +2539,45 @@
     </row>
     <row r="5" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="12"/>
-      <c r="B5" s="119"/>
-      <c r="C5" s="119"/>
-      <c r="D5" s="119"/>
-      <c r="E5" s="119"/>
-      <c r="F5" s="119"/>
-      <c r="G5" s="119"/>
-      <c r="H5" s="119"/>
-      <c r="I5" s="119"/>
-      <c r="J5" s="119"/>
-      <c r="K5" s="119"/>
-      <c r="L5" s="119"/>
+      <c r="B5" s="136"/>
+      <c r="C5" s="136"/>
+      <c r="D5" s="136"/>
+      <c r="E5" s="136"/>
+      <c r="F5" s="136"/>
+      <c r="G5" s="136"/>
+      <c r="H5" s="136"/>
+      <c r="I5" s="136"/>
+      <c r="J5" s="136"/>
+      <c r="K5" s="136"/>
+      <c r="L5" s="136"/>
       <c r="M5" s="14"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="99"/>
-      <c r="P5" s="99"/>
-      <c r="Q5" s="99"/>
-      <c r="R5" s="99"/>
-      <c r="S5" s="99"/>
-      <c r="T5" s="99"/>
-      <c r="U5" s="99"/>
-      <c r="V5" s="99"/>
-      <c r="W5" s="99"/>
-      <c r="X5" s="99"/>
-      <c r="Y5" s="99"/>
-      <c r="Z5" s="99"/>
-      <c r="AA5" s="99"/>
-      <c r="AB5" s="99"/>
+      <c r="N5" s="102"/>
+      <c r="O5" s="102"/>
+      <c r="P5" s="102"/>
+      <c r="Q5" s="102"/>
+      <c r="R5" s="102"/>
+      <c r="S5" s="102"/>
+      <c r="T5" s="102"/>
+      <c r="U5" s="102"/>
+      <c r="V5" s="102"/>
+      <c r="W5" s="102"/>
+      <c r="X5" s="102"/>
+      <c r="Y5" s="102"/>
+      <c r="Z5" s="102"/>
+      <c r="AA5" s="102"/>
+      <c r="AB5" s="102"/>
       <c r="AC5" s="33"/>
-      <c r="AD5" s="119"/>
-      <c r="AE5" s="119"/>
-      <c r="AF5" s="119"/>
-      <c r="AG5" s="119"/>
-      <c r="AH5" s="119"/>
-      <c r="AI5" s="119"/>
-      <c r="AJ5" s="119"/>
-      <c r="AK5" s="119"/>
-      <c r="AL5" s="119"/>
-      <c r="AM5" s="119"/>
-      <c r="AN5" s="119"/>
+      <c r="AD5" s="136"/>
+      <c r="AE5" s="136"/>
+      <c r="AF5" s="136"/>
+      <c r="AG5" s="136"/>
+      <c r="AH5" s="136"/>
+      <c r="AI5" s="136"/>
+      <c r="AJ5" s="136"/>
+      <c r="AK5" s="136"/>
+      <c r="AL5" s="136"/>
+      <c r="AM5" s="136"/>
+      <c r="AN5" s="136"/>
       <c r="AO5" s="12"/>
       <c r="AP5" s="12"/>
       <c r="AQ5" s="12"/>
@@ -2685,11 +2722,11 @@
       <c r="AE8" s="82"/>
       <c r="AF8" s="83"/>
       <c r="AG8" s="35"/>
-      <c r="AH8" s="122" t="s">
+      <c r="AH8" s="139" t="s">
         <v>85</v>
       </c>
-      <c r="AI8" s="123"/>
-      <c r="AJ8" s="124"/>
+      <c r="AI8" s="140"/>
+      <c r="AJ8" s="141"/>
       <c r="AK8" s="37"/>
       <c r="AL8" s="81" t="s">
         <v>12</v>
@@ -2742,11 +2779,11 @@
       <c r="AI9" s="66"/>
       <c r="AJ9" s="67"/>
       <c r="AK9" s="43"/>
-      <c r="AL9" s="106" t="s">
+      <c r="AL9" s="105" t="s">
         <v>15</v>
       </c>
-      <c r="AM9" s="107"/>
-      <c r="AN9" s="108"/>
+      <c r="AM9" s="106"/>
+      <c r="AN9" s="107"/>
       <c r="AP9" s="46" t="s">
         <v>11</v>
       </c>
@@ -2793,11 +2830,11 @@
       <c r="AI10" s="85"/>
       <c r="AJ10" s="86"/>
       <c r="AK10" s="44"/>
-      <c r="AL10" s="133" t="s">
+      <c r="AL10" s="148" t="s">
         <v>96</v>
       </c>
-      <c r="AM10" s="134"/>
-      <c r="AN10" s="135"/>
+      <c r="AM10" s="149"/>
+      <c r="AN10" s="150"/>
       <c r="AP10" s="46" t="s">
         <v>8</v>
       </c>
@@ -2863,10 +2900,10 @@
       <c r="C12" s="64"/>
       <c r="D12" s="57"/>
       <c r="E12" s="39"/>
-      <c r="F12" s="102" t="s">
+      <c r="F12" s="113" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="103"/>
+      <c r="G12" s="114"/>
       <c r="H12" s="59" t="s">
         <v>69</v>
       </c>
@@ -3028,11 +3065,11 @@
       <c r="C15" s="66"/>
       <c r="D15" s="67"/>
       <c r="E15" s="44"/>
-      <c r="F15" s="106" t="s">
+      <c r="F15" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="107"/>
-      <c r="H15" s="108"/>
+      <c r="G15" s="106"/>
+      <c r="H15" s="107"/>
       <c r="I15" s="43"/>
       <c r="J15" s="65"/>
       <c r="K15" s="66"/>
@@ -3072,7 +3109,7 @@
       </c>
       <c r="AQ15" s="25">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AR15" s="30"/>
     </row>
@@ -3081,11 +3118,11 @@
       <c r="C16" s="85"/>
       <c r="D16" s="86"/>
       <c r="E16" s="44"/>
-      <c r="F16" s="133" t="s">
+      <c r="F16" s="148" t="s">
         <v>88</v>
       </c>
-      <c r="G16" s="134"/>
-      <c r="H16" s="135"/>
+      <c r="G16" s="149"/>
+      <c r="H16" s="150"/>
       <c r="I16" s="44"/>
       <c r="J16" s="84"/>
       <c r="K16" s="85"/>
@@ -3123,7 +3160,7 @@
       </c>
       <c r="AQ16" s="25">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR16" s="30"/>
     </row>
@@ -3189,23 +3226,23 @@
       <c r="K18" s="33"/>
       <c r="L18" s="33"/>
       <c r="M18" s="5"/>
-      <c r="N18" s="99" t="s">
+      <c r="N18" s="102" t="s">
         <v>59</v>
       </c>
-      <c r="O18" s="99"/>
-      <c r="P18" s="99"/>
-      <c r="Q18" s="99"/>
-      <c r="R18" s="99"/>
-      <c r="S18" s="99"/>
-      <c r="T18" s="99"/>
-      <c r="U18" s="99"/>
-      <c r="V18" s="99"/>
-      <c r="W18" s="99"/>
-      <c r="X18" s="99"/>
-      <c r="Y18" s="99"/>
-      <c r="Z18" s="99"/>
-      <c r="AA18" s="99"/>
-      <c r="AB18" s="99"/>
+      <c r="O18" s="102"/>
+      <c r="P18" s="102"/>
+      <c r="Q18" s="102"/>
+      <c r="R18" s="102"/>
+      <c r="S18" s="102"/>
+      <c r="T18" s="102"/>
+      <c r="U18" s="102"/>
+      <c r="V18" s="102"/>
+      <c r="W18" s="102"/>
+      <c r="X18" s="102"/>
+      <c r="Y18" s="102"/>
+      <c r="Z18" s="102"/>
+      <c r="AA18" s="102"/>
+      <c r="AB18" s="102"/>
       <c r="AC18" s="33"/>
       <c r="AD18" s="33"/>
       <c r="AE18" s="33"/>
@@ -3240,21 +3277,21 @@
       <c r="K19" s="33"/>
       <c r="L19" s="33"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="99"/>
-      <c r="O19" s="99"/>
-      <c r="P19" s="99"/>
-      <c r="Q19" s="99"/>
-      <c r="R19" s="99"/>
-      <c r="S19" s="99"/>
-      <c r="T19" s="99"/>
-      <c r="U19" s="99"/>
-      <c r="V19" s="99"/>
-      <c r="W19" s="99"/>
-      <c r="X19" s="99"/>
-      <c r="Y19" s="99"/>
-      <c r="Z19" s="99"/>
-      <c r="AA19" s="99"/>
-      <c r="AB19" s="99"/>
+      <c r="N19" s="102"/>
+      <c r="O19" s="102"/>
+      <c r="P19" s="102"/>
+      <c r="Q19" s="102"/>
+      <c r="R19" s="102"/>
+      <c r="S19" s="102"/>
+      <c r="T19" s="102"/>
+      <c r="U19" s="102"/>
+      <c r="V19" s="102"/>
+      <c r="W19" s="102"/>
+      <c r="X19" s="102"/>
+      <c r="Y19" s="102"/>
+      <c r="Z19" s="102"/>
+      <c r="AA19" s="102"/>
+      <c r="AB19" s="102"/>
       <c r="AC19" s="33"/>
       <c r="AD19" s="33"/>
       <c r="AE19" s="33"/>
@@ -3272,7 +3309,7 @@
       </c>
       <c r="AQ19" s="25">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AR19" s="30"/>
     </row>
@@ -3289,18 +3326,18 @@
       <c r="K20" s="64"/>
       <c r="L20" s="57"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="136" t="s">
+      <c r="N20" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="O20" s="137"/>
+      <c r="O20" s="112"/>
       <c r="P20" s="60" t="s">
         <v>49</v>
       </c>
       <c r="Q20" s="39"/>
-      <c r="R20" s="136" t="s">
+      <c r="R20" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="S20" s="137"/>
+      <c r="S20" s="112"/>
       <c r="T20" s="60" t="s">
         <v>49</v>
       </c>
@@ -3354,16 +3391,16 @@
       <c r="K21" s="69"/>
       <c r="L21" s="61"/>
       <c r="M21" s="15"/>
-      <c r="N21" s="131" t="s">
+      <c r="N21" s="108" t="s">
         <v>92</v>
       </c>
-      <c r="O21" s="132"/>
+      <c r="O21" s="109"/>
       <c r="P21" s="62"/>
       <c r="Q21" s="36"/>
-      <c r="R21" s="131" t="s">
+      <c r="R21" s="108" t="s">
         <v>92</v>
       </c>
-      <c r="S21" s="132"/>
+      <c r="S21" s="109"/>
       <c r="T21" s="62"/>
       <c r="U21" s="36"/>
       <c r="V21" s="89" t="s">
@@ -3411,17 +3448,17 @@
       <c r="K22" s="82"/>
       <c r="L22" s="83"/>
       <c r="M22" s="4"/>
-      <c r="N22" s="125" t="s">
+      <c r="N22" s="142" t="s">
         <v>97</v>
       </c>
-      <c r="O22" s="126"/>
-      <c r="P22" s="127"/>
+      <c r="O22" s="143"/>
+      <c r="P22" s="144"/>
       <c r="Q22" s="35"/>
-      <c r="R22" s="125" t="s">
+      <c r="R22" s="142" t="s">
         <v>98</v>
       </c>
-      <c r="S22" s="126"/>
-      <c r="T22" s="127"/>
+      <c r="S22" s="143"/>
+      <c r="T22" s="144"/>
       <c r="U22" s="37"/>
       <c r="V22" s="81" t="s">
         <v>12</v>
@@ -3437,11 +3474,11 @@
       <c r="AE22" s="82"/>
       <c r="AF22" s="83"/>
       <c r="AG22" s="35"/>
-      <c r="AH22" s="122" t="s">
+      <c r="AH22" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="AI22" s="123"/>
-      <c r="AJ22" s="124"/>
+      <c r="AI22" s="140"/>
+      <c r="AJ22" s="141"/>
       <c r="AK22" s="37"/>
       <c r="AL22" s="81"/>
       <c r="AM22" s="82"/>
@@ -3468,13 +3505,13 @@
       <c r="K23" s="85"/>
       <c r="L23" s="86"/>
       <c r="M23" s="4"/>
-      <c r="N23" s="128"/>
-      <c r="O23" s="129"/>
-      <c r="P23" s="130"/>
+      <c r="N23" s="145"/>
+      <c r="O23" s="146"/>
+      <c r="P23" s="147"/>
       <c r="Q23" s="44"/>
-      <c r="R23" s="128"/>
-      <c r="S23" s="129"/>
-      <c r="T23" s="130"/>
+      <c r="R23" s="145"/>
+      <c r="S23" s="146"/>
+      <c r="T23" s="147"/>
       <c r="U23" s="44"/>
       <c r="V23" s="84"/>
       <c r="W23" s="85"/>
@@ -3568,23 +3605,23 @@
       <c r="K25" s="33"/>
       <c r="L25" s="33"/>
       <c r="M25" s="4"/>
-      <c r="N25" s="99" t="s">
+      <c r="N25" s="102" t="s">
         <v>39</v>
       </c>
-      <c r="O25" s="99"/>
-      <c r="P25" s="99"/>
-      <c r="Q25" s="99"/>
-      <c r="R25" s="99"/>
-      <c r="S25" s="99"/>
-      <c r="T25" s="99"/>
-      <c r="U25" s="99"/>
-      <c r="V25" s="99"/>
-      <c r="W25" s="99"/>
-      <c r="X25" s="99"/>
-      <c r="Y25" s="99"/>
-      <c r="Z25" s="99"/>
-      <c r="AA25" s="99"/>
-      <c r="AB25" s="99"/>
+      <c r="O25" s="102"/>
+      <c r="P25" s="102"/>
+      <c r="Q25" s="102"/>
+      <c r="R25" s="102"/>
+      <c r="S25" s="102"/>
+      <c r="T25" s="102"/>
+      <c r="U25" s="102"/>
+      <c r="V25" s="102"/>
+      <c r="W25" s="102"/>
+      <c r="X25" s="102"/>
+      <c r="Y25" s="102"/>
+      <c r="Z25" s="102"/>
+      <c r="AA25" s="102"/>
+      <c r="AB25" s="102"/>
       <c r="AC25" s="33"/>
       <c r="AD25" s="33"/>
       <c r="AE25" s="33"/>
@@ -3619,21 +3656,21 @@
       <c r="K26" s="33"/>
       <c r="L26" s="33"/>
       <c r="M26" s="4"/>
-      <c r="N26" s="99"/>
-      <c r="O26" s="99"/>
-      <c r="P26" s="99"/>
-      <c r="Q26" s="99"/>
-      <c r="R26" s="99"/>
-      <c r="S26" s="99"/>
-      <c r="T26" s="99"/>
-      <c r="U26" s="99"/>
-      <c r="V26" s="99"/>
-      <c r="W26" s="99"/>
-      <c r="X26" s="99"/>
-      <c r="Y26" s="99"/>
-      <c r="Z26" s="99"/>
-      <c r="AA26" s="99"/>
-      <c r="AB26" s="99"/>
+      <c r="N26" s="102"/>
+      <c r="O26" s="102"/>
+      <c r="P26" s="102"/>
+      <c r="Q26" s="102"/>
+      <c r="R26" s="102"/>
+      <c r="S26" s="102"/>
+      <c r="T26" s="102"/>
+      <c r="U26" s="102"/>
+      <c r="V26" s="102"/>
+      <c r="W26" s="102"/>
+      <c r="X26" s="102"/>
+      <c r="Y26" s="102"/>
+      <c r="Z26" s="102"/>
+      <c r="AA26" s="102"/>
+      <c r="AB26" s="102"/>
       <c r="AC26" s="33"/>
       <c r="AD26" s="33"/>
       <c r="AE26" s="33"/>
@@ -3674,16 +3711,16 @@
       <c r="O27" s="88"/>
       <c r="P27" s="34"/>
       <c r="Q27" s="36"/>
-      <c r="R27" s="104"/>
-      <c r="S27" s="105"/>
+      <c r="R27" s="121"/>
+      <c r="S27" s="122"/>
       <c r="T27" s="55"/>
       <c r="U27" s="36"/>
-      <c r="V27" s="104"/>
-      <c r="W27" s="105"/>
+      <c r="V27" s="121"/>
+      <c r="W27" s="122"/>
       <c r="X27" s="55"/>
       <c r="Y27" s="36"/>
-      <c r="Z27" s="104"/>
-      <c r="AA27" s="105"/>
+      <c r="Z27" s="121"/>
+      <c r="AA27" s="122"/>
       <c r="AB27" s="55"/>
       <c r="AC27" s="36"/>
       <c r="AD27" s="87" t="s">
@@ -3739,12 +3776,12 @@
       <c r="S28" s="90"/>
       <c r="T28" s="18"/>
       <c r="U28" s="38"/>
-      <c r="V28" s="100"/>
-      <c r="W28" s="101"/>
+      <c r="V28" s="103"/>
+      <c r="W28" s="104"/>
       <c r="X28" s="56"/>
       <c r="Y28" s="36"/>
-      <c r="Z28" s="100"/>
-      <c r="AA28" s="101"/>
+      <c r="Z28" s="103"/>
+      <c r="AA28" s="104"/>
       <c r="AB28" s="56"/>
       <c r="AC28" s="36"/>
       <c r="AD28" s="89"/>
@@ -3768,54 +3805,54 @@
       <c r="AR28" s="30"/>
     </row>
     <row r="29" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="95"/>
-      <c r="C29" s="96"/>
+      <c r="B29" s="98"/>
+      <c r="C29" s="99"/>
       <c r="D29" s="41"/>
       <c r="E29" s="37"/>
-      <c r="F29" s="95"/>
-      <c r="G29" s="96"/>
+      <c r="F29" s="98"/>
+      <c r="G29" s="99"/>
       <c r="H29" s="41"/>
       <c r="I29" s="35"/>
-      <c r="J29" s="95"/>
-      <c r="K29" s="96"/>
+      <c r="J29" s="98"/>
+      <c r="K29" s="99"/>
       <c r="L29" s="41"/>
       <c r="M29" s="5"/>
-      <c r="N29" s="95"/>
-      <c r="O29" s="96"/>
+      <c r="N29" s="98"/>
+      <c r="O29" s="99"/>
       <c r="P29" s="41"/>
       <c r="Q29" s="35"/>
-      <c r="R29" s="95"/>
-      <c r="S29" s="96"/>
+      <c r="R29" s="98"/>
+      <c r="S29" s="99"/>
       <c r="T29" s="41"/>
       <c r="U29" s="37"/>
-      <c r="V29" s="95"/>
-      <c r="W29" s="96"/>
+      <c r="V29" s="98"/>
+      <c r="W29" s="99"/>
       <c r="X29" s="41"/>
       <c r="Y29" s="35"/>
-      <c r="Z29" s="95"/>
-      <c r="AA29" s="96"/>
+      <c r="Z29" s="98"/>
+      <c r="AA29" s="99"/>
       <c r="AB29" s="41"/>
       <c r="AC29" s="35"/>
-      <c r="AD29" s="95" t="s">
+      <c r="AD29" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="AE29" s="96"/>
+      <c r="AE29" s="99"/>
       <c r="AF29" s="41" t="s">
         <v>32</v>
       </c>
       <c r="AG29" s="37"/>
-      <c r="AH29" s="95" t="s">
+      <c r="AH29" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="AI29" s="96"/>
+      <c r="AI29" s="99"/>
       <c r="AJ29" s="41" t="s">
         <v>32</v>
       </c>
       <c r="AK29" s="35"/>
-      <c r="AL29" s="95" t="s">
+      <c r="AL29" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="AM29" s="96"/>
+      <c r="AM29" s="99"/>
       <c r="AN29" s="41" t="s">
         <v>32</v>
       </c>
@@ -3829,54 +3866,54 @@
       <c r="AR29" s="30"/>
     </row>
     <row r="30" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="97"/>
-      <c r="C30" s="98"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="101"/>
       <c r="D30" s="45"/>
       <c r="E30" s="43"/>
-      <c r="F30" s="97"/>
-      <c r="G30" s="98"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="101"/>
       <c r="H30" s="45"/>
       <c r="I30" s="43"/>
-      <c r="J30" s="97"/>
-      <c r="K30" s="98"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="101"/>
       <c r="L30" s="45"/>
       <c r="M30" s="5"/>
-      <c r="N30" s="97"/>
-      <c r="O30" s="98"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="101"/>
       <c r="P30" s="45"/>
       <c r="Q30" s="43"/>
-      <c r="R30" s="97"/>
-      <c r="S30" s="98"/>
+      <c r="R30" s="100"/>
+      <c r="S30" s="101"/>
       <c r="T30" s="45"/>
       <c r="U30" s="43"/>
-      <c r="V30" s="97"/>
-      <c r="W30" s="98"/>
+      <c r="V30" s="100"/>
+      <c r="W30" s="101"/>
       <c r="X30" s="45"/>
       <c r="Y30" s="43"/>
-      <c r="Z30" s="97"/>
-      <c r="AA30" s="98"/>
+      <c r="Z30" s="100"/>
+      <c r="AA30" s="101"/>
       <c r="AB30" s="45"/>
       <c r="AC30" s="43"/>
-      <c r="AD30" s="97" t="s">
+      <c r="AD30" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="AE30" s="98"/>
+      <c r="AE30" s="101"/>
       <c r="AF30" s="45" t="s">
         <v>33</v>
       </c>
       <c r="AG30" s="43"/>
-      <c r="AH30" s="97" t="s">
+      <c r="AH30" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="AI30" s="98"/>
+      <c r="AI30" s="101"/>
       <c r="AJ30" s="45" t="s">
         <v>33</v>
       </c>
       <c r="AK30" s="43"/>
-      <c r="AL30" s="97" t="s">
+      <c r="AL30" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="AM30" s="98"/>
+      <c r="AM30" s="101"/>
       <c r="AN30" s="45" t="s">
         <v>33</v>
       </c>
@@ -4152,23 +4189,23 @@
       <c r="K36" s="33"/>
       <c r="L36" s="33"/>
       <c r="M36" s="4"/>
-      <c r="N36" s="99" t="s">
+      <c r="N36" s="102" t="s">
         <v>36</v>
       </c>
-      <c r="O36" s="99"/>
-      <c r="P36" s="99"/>
-      <c r="Q36" s="99"/>
-      <c r="R36" s="99"/>
-      <c r="S36" s="99"/>
-      <c r="T36" s="99"/>
-      <c r="U36" s="99"/>
-      <c r="V36" s="99"/>
-      <c r="W36" s="99"/>
-      <c r="X36" s="99"/>
-      <c r="Y36" s="99"/>
-      <c r="Z36" s="99"/>
-      <c r="AA36" s="99"/>
-      <c r="AB36" s="99"/>
+      <c r="O36" s="102"/>
+      <c r="P36" s="102"/>
+      <c r="Q36" s="102"/>
+      <c r="R36" s="102"/>
+      <c r="S36" s="102"/>
+      <c r="T36" s="102"/>
+      <c r="U36" s="102"/>
+      <c r="V36" s="102"/>
+      <c r="W36" s="102"/>
+      <c r="X36" s="102"/>
+      <c r="Y36" s="102"/>
+      <c r="Z36" s="102"/>
+      <c r="AA36" s="102"/>
+      <c r="AB36" s="102"/>
       <c r="AC36" s="33"/>
       <c r="AD36" s="33"/>
       <c r="AE36" s="33"/>
@@ -4200,21 +4237,21 @@
       <c r="K37" s="33"/>
       <c r="L37" s="33"/>
       <c r="M37" s="5"/>
-      <c r="N37" s="99"/>
-      <c r="O37" s="99"/>
-      <c r="P37" s="99"/>
-      <c r="Q37" s="99"/>
-      <c r="R37" s="99"/>
-      <c r="S37" s="99"/>
-      <c r="T37" s="99"/>
-      <c r="U37" s="99"/>
-      <c r="V37" s="99"/>
-      <c r="W37" s="99"/>
-      <c r="X37" s="99"/>
-      <c r="Y37" s="99"/>
-      <c r="Z37" s="99"/>
-      <c r="AA37" s="99"/>
-      <c r="AB37" s="99"/>
+      <c r="N37" s="102"/>
+      <c r="O37" s="102"/>
+      <c r="P37" s="102"/>
+      <c r="Q37" s="102"/>
+      <c r="R37" s="102"/>
+      <c r="S37" s="102"/>
+      <c r="T37" s="102"/>
+      <c r="U37" s="102"/>
+      <c r="V37" s="102"/>
+      <c r="W37" s="102"/>
+      <c r="X37" s="102"/>
+      <c r="Y37" s="102"/>
+      <c r="Z37" s="102"/>
+      <c r="AA37" s="102"/>
+      <c r="AB37" s="102"/>
       <c r="AC37" s="33"/>
       <c r="AD37" s="33"/>
       <c r="AE37" s="33"/>
@@ -4468,11 +4505,11 @@
       <c r="AE41" s="66"/>
       <c r="AF41" s="67"/>
       <c r="AG41" s="37"/>
-      <c r="AH41" s="150" t="s">
-        <v>106</v>
-      </c>
-      <c r="AI41" s="151"/>
-      <c r="AJ41" s="152"/>
+      <c r="AH41" s="95" t="s">
+        <v>105</v>
+      </c>
+      <c r="AI41" s="96"/>
+      <c r="AJ41" s="97"/>
       <c r="AK41" s="31"/>
       <c r="AL41" s="65" t="s">
         <v>24</v>
@@ -4890,11 +4927,11 @@
       <c r="AI48" s="66"/>
       <c r="AJ48" s="67"/>
       <c r="AK48" s="44"/>
-      <c r="AL48" s="106" t="s">
-        <v>18</v>
-      </c>
-      <c r="AM48" s="107"/>
-      <c r="AN48" s="108"/>
+      <c r="AL48" s="105" t="s">
+        <v>10</v>
+      </c>
+      <c r="AM48" s="106"/>
+      <c r="AN48" s="107"/>
       <c r="AO48" s="31"/>
       <c r="AP48" s="31"/>
       <c r="AQ48" s="31"/>
@@ -4923,11 +4960,11 @@
       <c r="O49" s="66"/>
       <c r="P49" s="67"/>
       <c r="Q49" s="44"/>
-      <c r="R49" s="106" t="s">
+      <c r="R49" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="S49" s="107"/>
-      <c r="T49" s="108"/>
+      <c r="S49" s="106"/>
+      <c r="T49" s="107"/>
       <c r="U49" s="44"/>
       <c r="V49" s="65" t="s">
         <v>18</v>
@@ -4947,11 +4984,11 @@
       <c r="AE49" s="66"/>
       <c r="AF49" s="67"/>
       <c r="AG49" s="35"/>
-      <c r="AH49" s="150" t="s">
-        <v>105</v>
-      </c>
-      <c r="AI49" s="151"/>
-      <c r="AJ49" s="152"/>
+      <c r="AH49" s="65" t="s">
+        <v>15</v>
+      </c>
+      <c r="AI49" s="66"/>
+      <c r="AJ49" s="67"/>
       <c r="AK49" s="44"/>
       <c r="AL49" s="65" t="s">
         <v>26</v>
@@ -4986,11 +5023,11 @@
       <c r="O50" s="72"/>
       <c r="P50" s="73"/>
       <c r="Q50" s="50"/>
-      <c r="R50" s="147" t="s">
+      <c r="R50" s="160" t="s">
         <v>96</v>
       </c>
-      <c r="S50" s="148"/>
-      <c r="T50" s="149"/>
+      <c r="S50" s="161"/>
+      <c r="T50" s="162"/>
       <c r="U50" s="50"/>
       <c r="V50" s="65" t="s">
         <v>15</v>
@@ -5004,11 +5041,11 @@
       <c r="AA50" s="66"/>
       <c r="AB50" s="67"/>
       <c r="AC50" s="50"/>
-      <c r="AD50" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE50" s="72"/>
-      <c r="AF50" s="73"/>
+      <c r="AD50" s="160" t="s">
+        <v>108</v>
+      </c>
+      <c r="AE50" s="161"/>
+      <c r="AF50" s="162"/>
       <c r="AG50" s="50"/>
       <c r="AH50" s="71" t="s">
         <v>14</v>
@@ -5080,10 +5117,10 @@
       <c r="C52" s="64"/>
       <c r="D52" s="57"/>
       <c r="E52" s="36"/>
-      <c r="F52" s="102" t="s">
+      <c r="F52" s="113" t="s">
         <v>89</v>
       </c>
-      <c r="G52" s="103"/>
+      <c r="G52" s="114"/>
       <c r="H52" s="59" t="s">
         <v>90</v>
       </c>
@@ -5100,10 +5137,10 @@
       <c r="O52" s="88"/>
       <c r="P52" s="34"/>
       <c r="Q52" s="31"/>
-      <c r="R52" s="102" t="s">
+      <c r="R52" s="113" t="s">
         <v>89</v>
       </c>
-      <c r="S52" s="103"/>
+      <c r="S52" s="114"/>
       <c r="T52" s="59" t="s">
         <v>94</v>
       </c>
@@ -5116,18 +5153,18 @@
       <c r="AA52" s="35"/>
       <c r="AB52" s="35"/>
       <c r="AC52" s="36"/>
-      <c r="AD52" s="102" t="s">
+      <c r="AD52" s="113" t="s">
         <v>89</v>
       </c>
-      <c r="AE52" s="103"/>
+      <c r="AE52" s="114"/>
       <c r="AF52" s="59" t="s">
         <v>102</v>
       </c>
       <c r="AG52" s="36"/>
-      <c r="AH52" s="102" t="s">
+      <c r="AH52" s="113" t="s">
         <v>89</v>
       </c>
-      <c r="AI52" s="103"/>
+      <c r="AI52" s="114"/>
       <c r="AJ52" s="59" t="s">
         <v>90</v>
       </c>
@@ -5333,7 +5370,7 @@
       <c r="AF56" s="67"/>
       <c r="AG56" s="44"/>
       <c r="AH56" s="65" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="AI56" s="66"/>
       <c r="AJ56" s="67"/>
@@ -5352,11 +5389,11 @@
       <c r="G57" s="72"/>
       <c r="H57" s="73"/>
       <c r="I57" s="50"/>
-      <c r="J57" s="141" t="s">
+      <c r="J57" s="154" t="s">
         <v>8</v>
       </c>
-      <c r="K57" s="142"/>
-      <c r="L57" s="143"/>
+      <c r="K57" s="155"/>
+      <c r="L57" s="156"/>
       <c r="M57" s="5"/>
       <c r="N57" s="71"/>
       <c r="O57" s="72"/>
@@ -5460,10 +5497,10 @@
       <c r="AA59" s="88"/>
       <c r="AB59" s="34"/>
       <c r="AC59" s="32"/>
-      <c r="AD59" s="102" t="s">
+      <c r="AD59" s="113" t="s">
         <v>89</v>
       </c>
-      <c r="AE59" s="103"/>
+      <c r="AE59" s="114"/>
       <c r="AF59" s="59" t="s">
         <v>90</v>
       </c>
@@ -5761,16 +5798,16 @@
       <c r="S66" s="88"/>
       <c r="T66" s="34"/>
       <c r="U66" s="36"/>
-      <c r="V66" s="102" t="s">
+      <c r="V66" s="111" t="s">
         <v>99</v>
       </c>
-      <c r="W66" s="103"/>
-      <c r="X66" s="59"/>
+      <c r="W66" s="112"/>
+      <c r="X66" s="60"/>
       <c r="Y66" s="36"/>
-      <c r="Z66" s="102" t="s">
+      <c r="Z66" s="113" t="s">
         <v>99</v>
       </c>
-      <c r="AA66" s="103"/>
+      <c r="AA66" s="114"/>
       <c r="AB66" s="59"/>
       <c r="AC66" s="36"/>
       <c r="AD66" s="87"/>
@@ -5811,11 +5848,11 @@
       <c r="S67" s="93"/>
       <c r="T67" s="94"/>
       <c r="U67" s="36"/>
-      <c r="V67" s="92" t="s">
+      <c r="V67" s="115" t="s">
         <v>100</v>
       </c>
-      <c r="W67" s="93"/>
-      <c r="X67" s="94"/>
+      <c r="W67" s="116"/>
+      <c r="X67" s="117"/>
       <c r="Y67" s="36"/>
       <c r="Z67" s="92" t="s">
         <v>100</v>
@@ -5861,9 +5898,11 @@
       <c r="S68" s="90"/>
       <c r="T68" s="91"/>
       <c r="U68" s="43"/>
-      <c r="V68" s="89"/>
-      <c r="W68" s="90"/>
-      <c r="X68" s="91"/>
+      <c r="V68" s="108" t="s">
+        <v>92</v>
+      </c>
+      <c r="W68" s="109"/>
+      <c r="X68" s="110"/>
       <c r="Y68" s="43"/>
       <c r="Z68" s="89"/>
       <c r="AA68" s="90"/>
@@ -5909,11 +5948,11 @@
       <c r="S69" s="66"/>
       <c r="T69" s="67"/>
       <c r="U69" s="37"/>
-      <c r="V69" s="65" t="s">
-        <v>25</v>
-      </c>
-      <c r="W69" s="66"/>
-      <c r="X69" s="67"/>
+      <c r="V69" s="118" t="s">
+        <v>106</v>
+      </c>
+      <c r="W69" s="119"/>
+      <c r="X69" s="120"/>
       <c r="Y69" s="35"/>
       <c r="Z69" s="65" t="s">
         <v>22</v>
@@ -5961,14 +6000,14 @@
       <c r="S70" s="66"/>
       <c r="T70" s="67"/>
       <c r="U70" s="44"/>
-      <c r="V70" s="65" t="s">
-        <v>24</v>
-      </c>
-      <c r="W70" s="66"/>
-      <c r="X70" s="67"/>
+      <c r="V70" s="118" t="s">
+        <v>107</v>
+      </c>
+      <c r="W70" s="119"/>
+      <c r="X70" s="120"/>
       <c r="Y70" s="40"/>
       <c r="Z70" s="65" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="AA70" s="66"/>
       <c r="AB70" s="67"/>
@@ -6013,15 +6052,17 @@
       <c r="S71" s="72"/>
       <c r="T71" s="73"/>
       <c r="U71" s="44"/>
-      <c r="V71" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="W71" s="72"/>
-      <c r="X71" s="73"/>
+      <c r="V71" s="123" t="s">
+        <v>108</v>
+      </c>
+      <c r="W71" s="124"/>
+      <c r="X71" s="125"/>
       <c r="Y71" s="44"/>
-      <c r="Z71" s="71"/>
-      <c r="AA71" s="72"/>
-      <c r="AB71" s="73"/>
+      <c r="Z71" s="160" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA71" s="161"/>
+      <c r="AB71" s="162"/>
       <c r="AC71" s="50"/>
       <c r="AD71" s="71"/>
       <c r="AE71" s="72"/>
@@ -6101,23 +6142,23 @@
       <c r="K73" s="33"/>
       <c r="L73" s="33"/>
       <c r="M73" s="14"/>
-      <c r="N73" s="99" t="s">
+      <c r="N73" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="O73" s="99"/>
-      <c r="P73" s="99"/>
-      <c r="Q73" s="99"/>
-      <c r="R73" s="99"/>
-      <c r="S73" s="99"/>
-      <c r="T73" s="99"/>
-      <c r="U73" s="99"/>
-      <c r="V73" s="99"/>
-      <c r="W73" s="99"/>
-      <c r="X73" s="99"/>
-      <c r="Y73" s="99"/>
-      <c r="Z73" s="99"/>
-      <c r="AA73" s="99"/>
-      <c r="AB73" s="99"/>
+      <c r="O73" s="102"/>
+      <c r="P73" s="102"/>
+      <c r="Q73" s="102"/>
+      <c r="R73" s="102"/>
+      <c r="S73" s="102"/>
+      <c r="T73" s="102"/>
+      <c r="U73" s="102"/>
+      <c r="V73" s="102"/>
+      <c r="W73" s="102"/>
+      <c r="X73" s="102"/>
+      <c r="Y73" s="102"/>
+      <c r="Z73" s="102"/>
+      <c r="AA73" s="102"/>
+      <c r="AB73" s="102"/>
       <c r="AD73" s="40"/>
       <c r="AE73" s="33"/>
       <c r="AF73" s="33"/>
@@ -6148,21 +6189,21 @@
       <c r="K74" s="33"/>
       <c r="L74" s="33"/>
       <c r="M74" s="14"/>
-      <c r="N74" s="99"/>
-      <c r="O74" s="99"/>
-      <c r="P74" s="99"/>
-      <c r="Q74" s="99"/>
-      <c r="R74" s="99"/>
-      <c r="S74" s="99"/>
-      <c r="T74" s="99"/>
-      <c r="U74" s="99"/>
-      <c r="V74" s="99"/>
-      <c r="W74" s="99"/>
-      <c r="X74" s="99"/>
-      <c r="Y74" s="99"/>
-      <c r="Z74" s="99"/>
-      <c r="AA74" s="99"/>
-      <c r="AB74" s="99"/>
+      <c r="N74" s="102"/>
+      <c r="O74" s="102"/>
+      <c r="P74" s="102"/>
+      <c r="Q74" s="102"/>
+      <c r="R74" s="102"/>
+      <c r="S74" s="102"/>
+      <c r="T74" s="102"/>
+      <c r="U74" s="102"/>
+      <c r="V74" s="102"/>
+      <c r="W74" s="102"/>
+      <c r="X74" s="102"/>
+      <c r="Y74" s="102"/>
+      <c r="Z74" s="102"/>
+      <c r="AA74" s="102"/>
+      <c r="AB74" s="102"/>
       <c r="AC74" s="21"/>
       <c r="AD74" s="33"/>
       <c r="AE74" s="33"/>
@@ -6182,16 +6223,16 @@
     </row>
     <row r="75" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="12"/>
-      <c r="B75" s="136" t="s">
+      <c r="B75" s="111" t="s">
         <v>58</v>
       </c>
-      <c r="C75" s="137"/>
+      <c r="C75" s="112"/>
       <c r="D75" s="60"/>
       <c r="E75" s="32"/>
-      <c r="F75" s="136" t="s">
+      <c r="F75" s="111" t="s">
         <v>52</v>
       </c>
-      <c r="G75" s="137"/>
+      <c r="G75" s="112"/>
       <c r="H75" s="60"/>
       <c r="I75" s="32"/>
       <c r="J75" s="63"/>
@@ -6252,17 +6293,17 @@
     </row>
     <row r="76" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="12"/>
-      <c r="B76" s="144" t="s">
+      <c r="B76" s="157" t="s">
         <v>92</v>
       </c>
-      <c r="C76" s="145"/>
-      <c r="D76" s="146"/>
+      <c r="C76" s="158"/>
+      <c r="D76" s="159"/>
       <c r="E76" s="32"/>
-      <c r="F76" s="144" t="s">
+      <c r="F76" s="157" t="s">
         <v>92</v>
       </c>
-      <c r="G76" s="145"/>
-      <c r="H76" s="146"/>
+      <c r="G76" s="158"/>
+      <c r="H76" s="159"/>
       <c r="I76" s="32"/>
       <c r="J76" s="78"/>
       <c r="K76" s="79"/>
@@ -6312,17 +6353,17 @@
     </row>
     <row r="77" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="16"/>
-      <c r="B77" s="138" t="s">
+      <c r="B77" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="C77" s="139"/>
-      <c r="D77" s="140"/>
+      <c r="C77" s="152"/>
+      <c r="D77" s="153"/>
       <c r="E77" s="32"/>
-      <c r="F77" s="138" t="s">
+      <c r="F77" s="151" t="s">
         <v>60</v>
       </c>
-      <c r="G77" s="139"/>
-      <c r="H77" s="140"/>
+      <c r="G77" s="152"/>
+      <c r="H77" s="153"/>
       <c r="I77" s="32"/>
       <c r="J77" s="68"/>
       <c r="K77" s="69"/>
@@ -6362,17 +6403,17 @@
     </row>
     <row r="78" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="16"/>
-      <c r="B78" s="125" t="s">
+      <c r="B78" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="C78" s="126"/>
-      <c r="D78" s="127"/>
+      <c r="C78" s="143"/>
+      <c r="D78" s="144"/>
       <c r="E78" s="32"/>
-      <c r="F78" s="125" t="s">
+      <c r="F78" s="142" t="s">
         <v>93</v>
       </c>
-      <c r="G78" s="126"/>
-      <c r="H78" s="127"/>
+      <c r="G78" s="143"/>
+      <c r="H78" s="144"/>
       <c r="I78" s="43"/>
       <c r="J78" s="81"/>
       <c r="K78" s="82"/>
@@ -6422,13 +6463,13 @@
     </row>
     <row r="79" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="16"/>
-      <c r="B79" s="128"/>
-      <c r="C79" s="129"/>
-      <c r="D79" s="130"/>
+      <c r="B79" s="145"/>
+      <c r="C79" s="146"/>
+      <c r="D79" s="147"/>
       <c r="E79" s="31"/>
-      <c r="F79" s="128"/>
-      <c r="G79" s="129"/>
-      <c r="H79" s="130"/>
+      <c r="F79" s="145"/>
+      <c r="G79" s="146"/>
+      <c r="H79" s="147"/>
       <c r="I79" s="32"/>
       <c r="J79" s="71"/>
       <c r="K79" s="72"/>
@@ -8276,6 +8317,7 @@
     <mergeCell ref="F107:H107"/>
     <mergeCell ref="J107:L107"/>
     <mergeCell ref="J109:L109"/>
+    <mergeCell ref="B112:D112"/>
     <mergeCell ref="B120:D120"/>
     <mergeCell ref="B121:D121"/>
     <mergeCell ref="B123:C123"/>
@@ -8290,7 +8332,6 @@
     <mergeCell ref="B115:D115"/>
     <mergeCell ref="F115:H115"/>
     <mergeCell ref="J115:L115"/>
-    <mergeCell ref="B112:D112"/>
     <mergeCell ref="F120:H120"/>
     <mergeCell ref="B126:D126"/>
     <mergeCell ref="F126:H126"/>
@@ -8556,6 +8597,10 @@
     <mergeCell ref="AH95:AJ95"/>
     <mergeCell ref="V90:X90"/>
     <mergeCell ref="V88:X88"/>
+    <mergeCell ref="R90:T90"/>
+    <mergeCell ref="AH88:AJ88"/>
+    <mergeCell ref="AH89:AJ89"/>
+    <mergeCell ref="AD85:AF85"/>
     <mergeCell ref="AL77:AN77"/>
     <mergeCell ref="AL78:AN78"/>
     <mergeCell ref="AD77:AF77"/>
@@ -8566,9 +8611,6 @@
     <mergeCell ref="AH81:AI81"/>
     <mergeCell ref="AL81:AM81"/>
     <mergeCell ref="AH78:AJ78"/>
-    <mergeCell ref="R83:T83"/>
-    <mergeCell ref="AD82:AF82"/>
-    <mergeCell ref="AH83:AJ83"/>
     <mergeCell ref="AD84:AF84"/>
     <mergeCell ref="AH84:AJ84"/>
     <mergeCell ref="AD83:AF83"/>
@@ -8586,10 +8628,6 @@
     <mergeCell ref="AD89:AF89"/>
     <mergeCell ref="AH87:AI87"/>
     <mergeCell ref="AL87:AM87"/>
-    <mergeCell ref="R90:T90"/>
-    <mergeCell ref="AH88:AJ88"/>
-    <mergeCell ref="AH89:AJ89"/>
-    <mergeCell ref="AD85:AF85"/>
     <mergeCell ref="AH85:AJ85"/>
     <mergeCell ref="AL85:AN85"/>
     <mergeCell ref="AH75:AI75"/>
@@ -8611,6 +8649,9 @@
     <mergeCell ref="V84:X84"/>
     <mergeCell ref="R82:T82"/>
     <mergeCell ref="V83:X83"/>
+    <mergeCell ref="R83:T83"/>
+    <mergeCell ref="AD82:AF82"/>
+    <mergeCell ref="AH83:AJ83"/>
     <mergeCell ref="N78:P78"/>
     <mergeCell ref="Z78:AB78"/>
     <mergeCell ref="N79:P79"/>
@@ -8725,7 +8766,6 @@
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="J30:K30"/>
     <mergeCell ref="J31:K31"/>
-    <mergeCell ref="J43:L43"/>
     <mergeCell ref="N47:P47"/>
     <mergeCell ref="F49:H49"/>
     <mergeCell ref="F46:H46"/>
@@ -8747,6 +8787,7 @@
     <mergeCell ref="J47:L47"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="J42:L42"/>
+    <mergeCell ref="F45:G45"/>
     <mergeCell ref="Z54:AB54"/>
     <mergeCell ref="Z50:AB50"/>
     <mergeCell ref="V45:W45"/>
@@ -8915,7 +8956,6 @@
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="J27:K27"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="F45:G45"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="F41:H41"/>
     <mergeCell ref="B41:D41"/>
@@ -8939,12 +8979,13 @@
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="F43:H43"/>
+    <mergeCell ref="J43:L43"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="D29:D34 AJ29:AJ34 X29:X34 T29:T34 AB29:AB34 AF29:AF34 P29:P34 H29:H34 L29:L34 AN29:AN34">
       <formula1>$AP$68:$AP$71</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="AL41:AN43 AH69:AJ71 AL90:AN91 J48:L50 N29:O34 Z29:AA34 F55:H57 J132:L133 V78:X79 R78:T79 AD96:AF97 Z56:AB57 R69:T71 Z78:AB79 Z48:AB51 Z96:AB97 B55:D57 AH48:AJ50 V8:X10 R101:T102 AD69:AF71 J114:L115 AL78:AN79 AL69:AN71 AH41:AJ43 R8:T10 B41:D43 B108:D109 B62:D64 Z14:AB16 AD41:AF43 R14:T16 F48:H50 AL14:AN16 F62:H64 J55:L57 N78:P79 R62:T64 B8:D10 J120:L121 F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 B126:D127 AD14:AF16 B114:D115 J126:L127 N48:P50 Z101:AB102 AD22:AF23 N84:P85 AD84:AF85 R22:T23 V14:X16 V22:X23 F108:H109 Z22:AB23 AL101:AN102 AL22:AN23 R55:T57 AD90:AF91 AD55:AF57 N22:P23 N90:P91 J22:L23 J62:L64 V48:X51 N96:P97 R84:T85 V96:X97 R41:T43 AD101:AF102 N14:P16 AD62:AF64 AH90:AJ91 V84:X85 Z41:AB43 AH62:AJ64 N101:P102 Z84:AB85 V41:X43 AH78:AJ79 AL84:AN85 AH55:AJ57 V56:X57 B29:C34 J29:K34 AH96:AJ97 AH101:AJ102 AL48:AN50 V90:X91 AL96:AN97 Z8:AB10 AH84:AJ85 AL8:AN10 N62:P64 N8:P10 AD78:AF79 V69:X71 AD8:AF10 V101:X102 V62:X64 AH8:AJ10 N55:P57 R29:S34 Z62:AB64 N41:P43 V29:W34 AL55:AN57 B78:D79 AL62:AN64 F29:G34 AD48:AF50 N69:P71 AL29:AM34 AH22:AJ23 AD29:AE34 AH29:AI34 R96:T97 AH14:AJ16 F22:H23 R90:T91 F8:H10 R48:T50 J8:L10 F14:H16 Z90:AB91 J14:L16 B14:D16 B22:D23 J41:L43 F69:H71 B69:D71 B48:D50 J69:L71 F41:H43 F78:H79 B96:D97 J78:L79 F84:H85 J101:L102 B84:D85 B101:D102 B90:D91 F96:H97 F101:H102 J90:L91 J96:L97 F90:H91 J84:L85 Z69:AB71">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="AL41:AN43 AH69:AJ71 AL90:AN91 J48:L50 N29:O34 Z29:AA34 F55:H57 J132:L133 V78:X79 R78:T79 AD96:AF97 Z56:AB57 R69:T71 Z78:AB79 Z48:AB51 Z96:AB97 B55:D57 AH55:AJ57 V8:X10 R101:T102 AD69:AF71 J114:L115 AL78:AN79 AL69:AN71 AH41:AJ43 R8:T10 B41:D43 B108:D109 B62:D64 Z14:AB16 AD41:AF43 R14:T16 F48:H50 AL14:AN16 F62:H64 J55:L57 N78:P79 R62:T64 B8:D10 J120:L121 F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 B126:D127 AD14:AF16 B114:D115 J126:L127 N48:P50 Z101:AB102 AD22:AF23 N84:P85 AD84:AF85 R22:T23 V14:X16 V22:X23 F108:H109 Z22:AB23 AL101:AN102 AL22:AN23 R55:T57 AD90:AF91 AD55:AF57 N22:P23 N90:P91 J22:L23 J62:L64 V48:X51 N96:P97 R84:T85 V96:X97 R41:T43 AD101:AF102 N14:P16 AD62:AF64 AH90:AJ91 V84:X85 Z41:AB43 AH62:AJ64 N101:P102 Z84:AB85 V41:X43 AH78:AJ79 AL84:AN85 AH48:AJ50 V56:X57 B29:C34 J29:K34 AH96:AJ97 AH101:AJ102 AL48:AN50 V90:X91 AL96:AN97 Z8:AB10 AH84:AJ85 AL8:AN10 N62:P64 N8:P10 AD78:AF79 V69:X71 AD8:AF10 V101:X102 V62:X64 AH8:AJ10 N55:P57 R29:S34 Z62:AB64 N41:P43 V29:W34 AL55:AN57 B78:D79 AL62:AN64 F29:G34 AD48:AF50 N69:P71 AL29:AM34 AH22:AJ23 AD29:AE34 AH29:AI34 R96:T97 AH14:AJ16 F22:H23 R90:T91 F8:H10 R48:T50 J8:L10 F14:H16 Z90:AB91 J14:L16 B14:D16 B22:D23 J41:L43 F69:H71 B69:D71 B48:D50 J69:L71 F41:H43 F78:H79 B96:D97 J78:L79 F84:H85 J101:L102 B84:D85 B101:D102 B90:D91 F96:H97 F101:H102 J90:L91 J96:L97 F90:H91 J84:L85 Z69:AB71">
       <formula1>$AP$6:$AP$30</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>